<commit_message>
Uploaded new emergency file
</commit_message>
<xml_diff>
--- a/Excel Portfolio Projects/Emergency Services Review/Emergency Services Review Project.xlsx
+++ b/Excel Portfolio Projects/Emergency Services Review/Emergency Services Review Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1ec44ccee5f08d5/Documents/Data Analysis/Portfolio/Excel Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="997" documentId="8_{88151A71-8DFA-4475-9035-398F879E8711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{433A7113-61FC-4808-A7F7-995CC0110388}"/>
+  <xr:revisionPtr revIDLastSave="1011" documentId="8_{88151A71-8DFA-4475-9035-398F879E8711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BE18E6F-A85F-4AC8-BBA9-D4A4B287A4DF}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-1790" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-1790" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Questions" sheetId="4" r:id="rId1"/>
@@ -348,10 +348,10 @@
       <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="0.0"/>
@@ -416,7 +416,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable4</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable4</c:name>
     <c:fmtId val="19"/>
   </c:pivotSource>
   <c:chart>
@@ -1469,7 +1469,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable5</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable5</c:name>
     <c:fmtId val="3"/>
   </c:pivotSource>
   <c:chart>
@@ -2579,7 +2579,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable3</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable3</c:name>
     <c:fmtId val="7"/>
   </c:pivotSource>
   <c:chart>
@@ -4339,7 +4339,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable6</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable6</c:name>
     <c:fmtId val="9"/>
   </c:pivotSource>
   <c:chart>
@@ -4654,13 +4654,13 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
               <a:spAutoFit/>
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1"/>
                   </a:solidFill>
@@ -4711,13 +4711,13 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
               <a:spAutoFit/>
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:sysClr val="windowText" lastClr="000000"/>
                   </a:solidFill>
@@ -6330,13 +6330,13 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1"/>
                     </a:solidFill>
@@ -6526,13 +6526,13 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:sysClr val="windowText" lastClr="000000"/>
                     </a:solidFill>
@@ -6861,7 +6861,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable2</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable2</c:name>
     <c:fmtId val="17"/>
   </c:pivotSource>
   <c:chart>
@@ -7043,7 +7043,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="bg1"/>
                   </a:solidFill>
@@ -8625,7 +8625,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="bg1"/>
                     </a:solidFill>
@@ -10307,7 +10307,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable18</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable18</c:name>
     <c:fmtId val="3"/>
   </c:pivotSource>
   <c:chart>
@@ -10850,7 +10850,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[UK_Public_Safety_Data_Project.xlsx]Raw Data!PivotTable19</c:name>
+    <c:name>[Emergency Services Review Project.xlsx]Raw Data!PivotTable19</c:name>
     <c:fmtId val="7"/>
   </c:pivotSource>
   <c:chart>
@@ -15977,7 +15977,7 @@
       <cdr:x>0.89742</cdr:x>
       <cdr:y>0.13203</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$29">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$28">
       <cdr:nvSpPr>
         <cdr:cNvPr id="18" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16098,7 +16098,7 @@
       <cdr:x>0.82085</cdr:x>
       <cdr:y>0.14201</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$28">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$27">
       <cdr:nvSpPr>
         <cdr:cNvPr id="33" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16219,7 +16219,7 @@
       <cdr:x>0.74243</cdr:x>
       <cdr:y>0.14502</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$27">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$26">
       <cdr:nvSpPr>
         <cdr:cNvPr id="34" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16340,7 +16340,7 @@
       <cdr:x>0.66648</cdr:x>
       <cdr:y>0.14202</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$26">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$25">
       <cdr:nvSpPr>
         <cdr:cNvPr id="35" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16461,7 +16461,7 @@
       <cdr:x>0.58639</cdr:x>
       <cdr:y>0.13769</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$25">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$24">
       <cdr:nvSpPr>
         <cdr:cNvPr id="38" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16582,7 +16582,7 @@
       <cdr:x>0.51225</cdr:x>
       <cdr:y>0.1261</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$24">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$23">
       <cdr:nvSpPr>
         <cdr:cNvPr id="37" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16703,7 +16703,7 @@
       <cdr:x>0.11512</cdr:x>
       <cdr:y>0.12038</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$19">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$18">
       <cdr:nvSpPr>
         <cdr:cNvPr id="39" name="TextBox 38">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16761,7 +16761,7 @@
       <cdr:x>0.19105</cdr:x>
       <cdr:y>0.13986</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$20">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$19">
       <cdr:nvSpPr>
         <cdr:cNvPr id="40" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -16883,7 +16883,7 @@
       <cdr:x>0.26759</cdr:x>
       <cdr:y>0.13527</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$21">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$20">
       <cdr:nvSpPr>
         <cdr:cNvPr id="41" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -17004,7 +17004,7 @@
       <cdr:x>0.97584</cdr:x>
       <cdr:y>0.12036</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$30">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$29">
       <cdr:nvSpPr>
         <cdr:cNvPr id="42" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -17125,7 +17125,7 @@
       <cdr:x>0.34972</cdr:x>
       <cdr:y>0.13266</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$22">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$21">
       <cdr:nvSpPr>
         <cdr:cNvPr id="43" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -17246,7 +17246,7 @@
       <cdr:x>0.42752</cdr:x>
       <cdr:y>0.13043</cdr:y>
     </cdr:to>
-    <cdr:sp macro="" textlink="'Raw Data'!$Y$23">
+    <cdr:sp macro="" textlink="'Raw Data'!$X$22">
       <cdr:nvSpPr>
         <cdr:cNvPr id="44" name="TextBox 1">
           <a:extLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -25413,6 +25413,143 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E32690AA-A4BE-4EA8-B960-10C58710362E}" name="PivotTable18" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="T33:U47" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="13">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="13">
+        <item x="7"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="6"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item x="4"/>
+        <item x="8"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="0"/>
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="14">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="7"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i r="1">
+      <x v="11"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Public Satisfaction (%)" fld="10" subtotal="average" baseField="0" baseItem="0" numFmtId="165"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="2">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="3" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="10"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5A0748F5-0DBB-4FCA-BA40-1AA3A02F43B4}" name="PivotTable2" cacheId="0" dataPosition="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="35">
   <location ref="O1:R28" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
@@ -26532,7 +26669,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7C55220A-B56C-4898-997C-ED31400853A5}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14">
   <location ref="O31:R40" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
@@ -26722,7 +26859,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70E5258A-CAC5-470F-A35B-D330CC354CE0}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="O43:R57" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="14">
@@ -26825,7 +26962,7 @@
     <dataField name="Average of Average Response Time (min)" fld="7" subtotal="average" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="7">
+    <format dxfId="8">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="0" count="1" selected="0">
@@ -26835,7 +26972,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="6">
+    <format dxfId="7">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="1">
@@ -26844,7 +26981,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="6">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="0" count="1" selected="0">
@@ -26854,10 +26991,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="4">
+    <format dxfId="5">
       <pivotArea grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="4">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="1">
@@ -26866,7 +27003,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="3">
       <pivotArea grandCol="1" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -26998,7 +27135,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{87152FF9-069B-4A5D-A601-9E3FB622E9C6}" name="PivotTable19" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
   <location ref="T49:U63" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="13">
@@ -27093,7 +27230,7 @@
     <dataField name="Average of Public Satisfaction (%)" fld="10" subtotal="average" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="8">
+    <format dxfId="9">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -27118,143 +27255,6 @@
           </reference>
           <reference field="1" count="1" selected="0">
             <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E32690AA-A4BE-4EA8-B960-10C58710362E}" name="PivotTable18" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="T33:U47" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="13">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item h="1" x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="13">
-        <item x="7"/>
-        <item x="9"/>
-        <item x="11"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="6"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="10"/>
-        <item x="4"/>
-        <item x="8"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="0"/>
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="14">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="7"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i r="1">
-      <x v="11"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Public Satisfaction (%)" fld="10" subtotal="average" baseField="0" baseItem="0" numFmtId="165"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="9">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="3" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="3">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="10"/>
           </reference>
         </references>
       </pivotArea>
@@ -27628,7 +27628,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y151"/>
+  <dimension ref="A1:X151"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -28705,7 +28705,7 @@
         <v>0.93158153904268515</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -28765,7 +28765,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -28830,8 +28830,12 @@
       <c r="W18" t="s">
         <v>42</v>
       </c>
+      <c r="X18">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","East Midlands")</f>
+        <v>1031</v>
+      </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -28896,12 +28900,12 @@
       <c r="W19" s="13">
         <v>1031</v>
       </c>
-      <c r="Y19">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","East Midlands")</f>
-        <v>1031</v>
+      <c r="X19">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","East of England")</f>
+        <v>2067</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -28966,12 +28970,12 @@
       <c r="W20">
         <v>2067</v>
       </c>
-      <c r="Y20">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","East of England")</f>
-        <v>2067</v>
+      <c r="X20">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","London")</f>
+        <v>1060</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -29036,12 +29040,12 @@
       <c r="W21">
         <v>1060</v>
       </c>
-      <c r="Y21">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","London")</f>
-        <v>1060</v>
+      <c r="X21">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","North East")</f>
+        <v>1592</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>25</v>
       </c>
@@ -29106,12 +29110,12 @@
       <c r="W22">
         <v>1592</v>
       </c>
-      <c r="Y22">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","North East")</f>
-        <v>1592</v>
+      <c r="X22">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","North West")</f>
+        <v>2049</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -29176,12 +29180,12 @@
       <c r="W23">
         <v>2049</v>
       </c>
-      <c r="Y23">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","North West")</f>
-        <v>2049</v>
+      <c r="X23">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Northern Ireland")</f>
+        <v>857</v>
       </c>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -29246,12 +29250,12 @@
       <c r="W24">
         <v>857</v>
       </c>
-      <c r="Y24">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Northern Ireland")</f>
-        <v>857</v>
+      <c r="X24">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Scotland")</f>
+        <v>1925</v>
       </c>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -29316,12 +29320,12 @@
       <c r="W25">
         <v>1925</v>
       </c>
-      <c r="Y25">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Scotland")</f>
-        <v>1925</v>
+      <c r="X25">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","South East")</f>
+        <v>1480</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -29386,12 +29390,12 @@
       <c r="W26">
         <v>1480</v>
       </c>
-      <c r="Y26">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","South East")</f>
-        <v>1480</v>
+      <c r="X26">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","South West")</f>
+        <v>1382</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -29456,12 +29460,12 @@
       <c r="W27">
         <v>1382</v>
       </c>
-      <c r="Y27">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","South West")</f>
-        <v>1382</v>
+      <c r="X27">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Wales")</f>
+        <v>1796</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -29526,12 +29530,12 @@
       <c r="W28">
         <v>1796</v>
       </c>
-      <c r="Y28">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Wales")</f>
-        <v>1796</v>
+      <c r="X28">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","West Midlands")</f>
+        <v>1756</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -29584,12 +29588,12 @@
       <c r="W29">
         <v>1756</v>
       </c>
-      <c r="Y29">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","West Midlands")</f>
-        <v>1756</v>
+      <c r="X29">
+        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Yorkshire and the Humber")</f>
+        <v>1234</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -29642,12 +29646,8 @@
       <c r="W30">
         <v>1234</v>
       </c>
-      <c r="Y30">
-        <f>GETPIVOTDATA("Staff Count",$T$17,"Region","Yorkshire and the Humber")</f>
-        <v>1234</v>
-      </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>25</v>
       </c>
@@ -29707,7 +29707,7 @@
         <v>18229</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -35650,17 +35650,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f7ad296a-57ff-428c-b4cb-07edbf36982d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2d161a28-3536-4ba6-9ad5-e5ce0dbbadc5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003B13CFFDAAE59C4CA678E7EE4E73178D" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e05d12ad55831ca1d94ab0d6bf4c33ae">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f7ad296a-57ff-428c-b4cb-07edbf36982d" xmlns:ns3="2d161a28-3536-4ba6-9ad5-e5ce0dbbadc5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="accd58e9f676c36d920d788803336cd6" ns2:_="" ns3:_="">
     <xsd:import namespace="f7ad296a-57ff-428c-b4cb-07edbf36982d"/>
@@ -35855,6 +35844,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f7ad296a-57ff-428c-b4cb-07edbf36982d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2d161a28-3536-4ba6-9ad5-e5ce0dbbadc5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1632C448-2796-4273-B186-9F60F8DD736F}">
   <ds:schemaRefs>
@@ -35864,23 +35864,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD253A9A-6DC7-4FA1-AF78-9A17C6B0F5FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="f7ad296a-57ff-428c-b4cb-07edbf36982d"/>
-    <ds:schemaRef ds:uri="2d161a28-3536-4ba6-9ad5-e5ce0dbbadc5"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E72BB855-D9E2-418E-8D59-E846EEFC1235}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -35897,4 +35880,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD253A9A-6DC7-4FA1-AF78-9A17C6B0F5FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="f7ad296a-57ff-428c-b4cb-07edbf36982d"/>
+    <ds:schemaRef ds:uri="2d161a28-3536-4ba6-9ad5-e5ce0dbbadc5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>